<commit_message>
docs: Actualiza avance de analisis de relaciones entre requisitos.
</commit_message>
<xml_diff>
--- a/docs/misc/project-work/StatPhi - Analisis de Relaciones entre Requisitos.xlsx
+++ b/docs/misc/project-work/StatPhi - Analisis de Relaciones entre Requisitos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonel\Desktop\Proyectos Programacion\JavaScript\statphi-backend\docs\misc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonel\Desktop\Proyectos Programacion\JavaScript\statphi-backend\docs\misc\project-work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{340E592A-D293-4B1A-86B0-E6D50E8333F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98A9850-95EF-4AFA-975E-D4FF48F33E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{E196C713-1D70-48E5-9163-96C2E2D36875}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="2" xr2:uid="{E196C713-1D70-48E5-9163-96C2E2D36875}"/>
   </bookViews>
   <sheets>
     <sheet name="Analisis Rel. Req." sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="390">
   <si>
     <t>ID</t>
   </si>
@@ -1156,6 +1156,63 @@
   </si>
   <si>
     <t>Para poder modificar o eliminar la foto de perfil de una cuenta (R104.8) antes se debe poder iniciar sesion (R104.2).</t>
+  </si>
+  <si>
+    <t>R118</t>
+  </si>
+  <si>
+    <t>R117</t>
+  </si>
+  <si>
+    <t>R116</t>
+  </si>
+  <si>
+    <t>Informar al usuario y bloquear las funciones asociadas a la conectividad (R117 y R118) requieren que las pruebas de conexión se puedan ejecutar (R116).</t>
+  </si>
+  <si>
+    <t>R121</t>
+  </si>
+  <si>
+    <t>R123</t>
+  </si>
+  <si>
+    <t>Para poder modificar la informacion del usuario (R121 y R123) antes se debe poder iniciar sesion (R104.2).</t>
+  </si>
+  <si>
+    <t>R125</t>
+  </si>
+  <si>
+    <t>R126</t>
+  </si>
+  <si>
+    <t>Para poder cerrar sesion (R125 y R126) antes se debe poder iniciar sesion (R104.2).</t>
+  </si>
+  <si>
+    <t>R127</t>
+  </si>
+  <si>
+    <t>Al modificar la informacion de acceso de la cuenta (R121) se aplica lo especificado en R127.</t>
+  </si>
+  <si>
+    <t>R128</t>
+  </si>
+  <si>
+    <t>R130</t>
+  </si>
+  <si>
+    <t>Antes de modificar la informacion personal de una cuenta (R121) o eliminarla (R130) se debe cumplir los especificado en R128.</t>
+  </si>
+  <si>
+    <t>R129</t>
+  </si>
+  <si>
+    <t>Cuando se cierre una sesion (R125 y R126) se debe aplicar lo especificado en R128.</t>
+  </si>
+  <si>
+    <t>Para poder cerrar un proyecto de una cuenta cargado en el sistema (R129) antes el sistema debe poder cargarlo (R104.5).</t>
+  </si>
+  <si>
+    <t>Para poder eliminar una cuenta (R130) antes debe estar creada (R104.1).</t>
   </si>
 </sst>
 </file>
@@ -1297,7 +1354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1352,7 +1409,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1364,22 +1430,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1388,10 +1451,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3322,7 +3382,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF41517A-2817-45FF-8D93-5F4C76EEC545}">
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="16"/>
@@ -3380,10 +3440,10 @@
       <c r="B4" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="24" t="s">
         <v>234</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="24" t="s">
         <v>235</v>
       </c>
     </row>
@@ -3394,8 +3454,8 @@
       <c r="B5" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
@@ -3460,7 +3520,7 @@
       <c r="B10" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="24" t="s">
         <v>58</v>
       </c>
       <c r="D10" s="8" t="s">
@@ -3474,8 +3534,8 @@
       <c r="B11" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="21" t="s">
+      <c r="C11" s="26"/>
+      <c r="D11" s="24" t="s">
         <v>226</v>
       </c>
     </row>
@@ -3486,8 +3546,8 @@
       <c r="B12" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
@@ -3496,8 +3556,8 @@
       <c r="B13" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
@@ -3506,8 +3566,8 @@
       <c r="B14" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
@@ -3516,8 +3576,8 @@
       <c r="B15" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
@@ -3526,8 +3586,8 @@
       <c r="B16" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
@@ -3536,8 +3596,8 @@
       <c r="B17" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
@@ -3546,8 +3606,8 @@
       <c r="B18" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
@@ -3556,8 +3616,8 @@
       <c r="B19" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="22"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="25"/>
     </row>
     <row r="20" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
@@ -3566,8 +3626,8 @@
       <c r="B20" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="20" t="s">
+      <c r="C20" s="26"/>
+      <c r="D20" s="27" t="s">
         <v>227</v>
       </c>
     </row>
@@ -3578,8 +3638,8 @@
       <c r="B21" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="20"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="27"/>
     </row>
     <row r="22" spans="1:4" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
@@ -3588,7 +3648,7 @@
       <c r="B22" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C22" s="22"/>
+      <c r="C22" s="25"/>
       <c r="D22" s="8" t="s">
         <v>229</v>
       </c>
@@ -3684,10 +3744,10 @@
       <c r="B29" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="C29" s="27" t="s">
         <v>247</v>
       </c>
-      <c r="D29" s="20" t="s">
+      <c r="D29" s="27" t="s">
         <v>250</v>
       </c>
     </row>
@@ -3698,8 +3758,8 @@
       <c r="B30" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
     </row>
     <row r="31" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
@@ -3708,10 +3768,10 @@
       <c r="B31" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="C31" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="24" t="s">
         <v>295</v>
       </c>
     </row>
@@ -3722,8 +3782,8 @@
       <c r="B32" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
@@ -3732,8 +3792,8 @@
       <c r="B33" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
     </row>
     <row r="34" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
@@ -3756,10 +3816,10 @@
       <c r="B35" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="27" t="s">
         <v>324</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="27" t="s">
         <v>255</v>
       </c>
     </row>
@@ -3770,8 +3830,8 @@
       <c r="B36" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
     </row>
     <row r="37" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
@@ -3780,8 +3840,8 @@
       <c r="B37" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
     </row>
     <row r="38" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
@@ -3790,10 +3850,10 @@
       <c r="B38" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C38" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="24" t="s">
         <v>304</v>
       </c>
     </row>
@@ -3804,8 +3864,8 @@
       <c r="B39" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
     </row>
     <row r="40" spans="1:4" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
@@ -3822,24 +3882,24 @@
       </c>
     </row>
     <row r="41" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="25" t="s">
+      <c r="A41" s="22" t="s">
         <v>300</v>
       </c>
-      <c r="B41" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="C41" s="21" t="s">
+      <c r="B41" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="C41" s="24" t="s">
         <v>297</v>
       </c>
-      <c r="D41" s="21" t="s">
+      <c r="D41" s="24" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="26"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
+      <c r="A42" s="23"/>
+      <c r="B42" s="25"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
     </row>
     <row r="43" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
@@ -3848,10 +3908,10 @@
       <c r="B43" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C43" s="20" t="s">
+      <c r="C43" s="27" t="s">
         <v>256</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D43" s="27" t="s">
         <v>257</v>
       </c>
     </row>
@@ -3862,8 +3922,8 @@
       <c r="B44" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
+      <c r="C44" s="27"/>
+      <c r="D44" s="27"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
@@ -3872,8 +3932,8 @@
       <c r="B45" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
@@ -3882,8 +3942,8 @@
       <c r="B46" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
@@ -3892,8 +3952,8 @@
       <c r="B47" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="27"/>
     </row>
     <row r="48" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
@@ -4050,7 +4110,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A59" s="24" t="s">
+      <c r="A59" s="21" t="s">
         <v>318</v>
       </c>
       <c r="B59" s="8" t="s">
@@ -4064,7 +4124,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A60" s="24"/>
+      <c r="A60" s="21"/>
       <c r="B60" s="8" t="s">
         <v>176</v>
       </c>
@@ -4082,10 +4142,10 @@
       <c r="B61" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C61" s="20" t="s">
+      <c r="C61" s="27" t="s">
         <v>318</v>
       </c>
-      <c r="D61" s="20" t="s">
+      <c r="D61" s="27" t="s">
         <v>327</v>
       </c>
     </row>
@@ -4096,8 +4156,8 @@
       <c r="B62" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C62" s="20"/>
-      <c r="D62" s="20"/>
+      <c r="C62" s="27"/>
+      <c r="D62" s="27"/>
     </row>
     <row r="63" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A63" s="15" t="s">
@@ -4134,7 +4194,7 @@
       <c r="B65" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="C65" s="24" t="s">
         <v>163</v>
       </c>
       <c r="D65" s="8" t="s">
@@ -4148,9 +4208,7 @@
       <c r="B66" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C66" s="21" t="s">
-        <v>163</v>
-      </c>
+      <c r="C66" s="26"/>
       <c r="D66" s="8" t="s">
         <v>367</v>
       </c>
@@ -4162,7 +4220,7 @@
       <c r="B67" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C67" s="23"/>
+      <c r="C67" s="26"/>
       <c r="D67" s="8" t="s">
         <v>369</v>
       </c>
@@ -4174,32 +4232,128 @@
       <c r="B68" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C68" s="22"/>
+      <c r="C68" s="26"/>
       <c r="D68" s="8" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
+        <v>375</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C69" s="26"/>
+      <c r="D69" s="24" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C70" s="26"/>
+      <c r="D70" s="25"/>
+    </row>
+    <row r="71" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="15" t="s">
+        <v>378</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C71" s="26"/>
+      <c r="D71" s="24" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="15" t="s">
+        <v>379</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C72" s="25"/>
+      <c r="D72" s="25"/>
+    </row>
+    <row r="73" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A73" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C73" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="D73" s="20" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A74" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="B69" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="C69" s="8" t="s">
+      <c r="B74" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C74" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="D69" s="8" t="s">
+      <c r="D74" s="8" t="s">
         <v>366</v>
       </c>
     </row>
+    <row r="75" spans="1:4" ht="135" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="15" t="s">
+        <v>372</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C75" s="27" t="s">
+        <v>373</v>
+      </c>
+      <c r="D75" s="27" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C76" s="27"/>
+      <c r="D76" s="27"/>
+    </row>
+    <row r="77" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A77" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>388</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C66:C68"/>
-    <mergeCell ref="D20:D21"/>
+  <mergeCells count="27">
+    <mergeCell ref="C75:C76"/>
+    <mergeCell ref="D75:D76"/>
+    <mergeCell ref="D69:D70"/>
+    <mergeCell ref="D71:D72"/>
+    <mergeCell ref="C65:C72"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="C35:C37"/>
@@ -4210,6 +4364,10 @@
     <mergeCell ref="C10:C22"/>
     <mergeCell ref="C31:C33"/>
     <mergeCell ref="D31:D33"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="D20:D21"/>
     <mergeCell ref="C38:C39"/>
     <mergeCell ref="D38:D39"/>
     <mergeCell ref="D41:D42"/>
@@ -4233,7 +4391,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A03B3C2-D12E-4478-B962-7F87C980A4EE}">
-  <dimension ref="A1:D111"/>
+  <dimension ref="A1:D116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="11"/>
@@ -4271,7 +4429,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="135" x14ac:dyDescent="0.25">
-      <c r="A3" s="32"/>
+      <c r="A3" s="29"/>
       <c r="B3" s="4" t="s">
         <v>176</v>
       </c>
@@ -4283,7 +4441,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A4" s="32"/>
+      <c r="A4" s="29"/>
       <c r="B4" s="4" t="s">
         <v>176</v>
       </c>
@@ -4295,7 +4453,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="150" x14ac:dyDescent="0.25">
-      <c r="A5" s="32"/>
+      <c r="A5" s="29"/>
       <c r="B5" s="4" t="s">
         <v>176</v>
       </c>
@@ -4307,7 +4465,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="135" x14ac:dyDescent="0.25">
-      <c r="A6" s="32"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="4" t="s">
         <v>176</v>
       </c>
@@ -4319,7 +4477,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A7" s="29"/>
+      <c r="A7" s="30"/>
       <c r="B7" s="4" t="s">
         <v>176</v>
       </c>
@@ -4345,7 +4503,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
+      <c r="A9" s="29"/>
       <c r="B9" s="4" t="s">
         <v>176</v>
       </c>
@@ -4357,7 +4515,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="29"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="4" t="s">
         <v>176</v>
       </c>
@@ -4375,10 +4533,10 @@
       <c r="B11" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="27" t="s">
         <v>187</v>
       </c>
     </row>
@@ -4389,8 +4547,8 @@
       <c r="B12" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="20"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -4399,10 +4557,10 @@
       <c r="B13" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="27" t="s">
         <v>188</v>
       </c>
     </row>
@@ -4413,8 +4571,8 @@
       <c r="B14" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="20"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="27"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -4423,8 +4581,8 @@
       <c r="B15" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="20"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="27"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -4433,10 +4591,10 @@
       <c r="B16" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="C16" s="27" t="s">
         <v>197</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="27" t="s">
         <v>284</v>
       </c>
     </row>
@@ -4447,8 +4605,8 @@
       <c r="B17" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
     </row>
     <row r="18" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
@@ -4457,10 +4615,10 @@
       <c r="B18" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="24" t="s">
         <v>222</v>
       </c>
     </row>
@@ -4471,8 +4629,8 @@
       <c r="B19" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
     </row>
     <row r="20" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="s">
@@ -4489,7 +4647,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
+      <c r="A21" s="29"/>
       <c r="B21" s="4" t="s">
         <v>176</v>
       </c>
@@ -4501,7 +4659,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
+      <c r="A22" s="29"/>
       <c r="B22" s="4" t="s">
         <v>176</v>
       </c>
@@ -4513,7 +4671,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
+      <c r="A23" s="29"/>
       <c r="B23" s="4" t="s">
         <v>176</v>
       </c>
@@ -4525,7 +4683,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A24" s="29"/>
+      <c r="A24" s="30"/>
       <c r="B24" s="4" t="s">
         <v>176</v>
       </c>
@@ -4543,10 +4701,10 @@
       <c r="B25" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C25" s="20" t="s">
+      <c r="C25" s="27" t="s">
         <v>201</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="27" t="s">
         <v>208</v>
       </c>
     </row>
@@ -4557,8 +4715,8 @@
       <c r="B26" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
@@ -4567,11 +4725,11 @@
       <c r="B27" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
     </row>
     <row r="28" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="34" t="s">
         <v>198</v>
       </c>
       <c r="B28" s="4" t="s">
@@ -4585,7 +4743,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A29" s="27"/>
+      <c r="A29" s="34"/>
       <c r="B29" s="4" t="s">
         <v>176</v>
       </c>
@@ -4597,7 +4755,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A30" s="27"/>
+      <c r="A30" s="34"/>
       <c r="B30" s="4" t="s">
         <v>176</v>
       </c>
@@ -4609,7 +4767,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A31" s="27"/>
+      <c r="A31" s="34"/>
       <c r="B31" s="4" t="s">
         <v>176</v>
       </c>
@@ -4621,7 +4779,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A32" s="27"/>
+      <c r="A32" s="34"/>
       <c r="B32" s="4" t="s">
         <v>176</v>
       </c>
@@ -4633,7 +4791,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A33" s="27"/>
+      <c r="A33" s="34"/>
       <c r="B33" s="4" t="s">
         <v>176</v>
       </c>
@@ -4665,10 +4823,10 @@
       <c r="B35" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="27" t="s">
         <v>232</v>
       </c>
-      <c r="D35" s="20" t="s">
+      <c r="D35" s="27" t="s">
         <v>233</v>
       </c>
     </row>
@@ -4679,8 +4837,8 @@
       <c r="B36" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="C36" s="27"/>
+      <c r="D36" s="27"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
@@ -4689,8 +4847,8 @@
       <c r="B37" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
+      <c r="C37" s="27"/>
+      <c r="D37" s="27"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
@@ -4699,8 +4857,8 @@
       <c r="B38" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
@@ -4709,8 +4867,8 @@
       <c r="B39" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -4719,8 +4877,8 @@
       <c r="B40" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
+      <c r="C40" s="27"/>
+      <c r="D40" s="27"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
@@ -4729,8 +4887,8 @@
       <c r="B41" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
+      <c r="C41" s="27"/>
+      <c r="D41" s="27"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
@@ -4739,8 +4897,8 @@
       <c r="B42" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="27"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
@@ -4749,8 +4907,8 @@
       <c r="B43" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="27"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
@@ -4759,8 +4917,8 @@
       <c r="B44" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
+      <c r="C44" s="27"/>
+      <c r="D44" s="27"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
@@ -4769,8 +4927,8 @@
       <c r="B45" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
+      <c r="C45" s="27"/>
+      <c r="D45" s="27"/>
     </row>
     <row r="46" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
@@ -4801,7 +4959,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A48" s="30" t="s">
+      <c r="A48" s="32" t="s">
         <v>101</v>
       </c>
       <c r="B48" s="8" t="s">
@@ -4815,7 +4973,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A49" s="31"/>
+      <c r="A49" s="33"/>
       <c r="B49" s="4" t="s">
         <v>176</v>
       </c>
@@ -4841,7 +4999,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A51" s="29"/>
+      <c r="A51" s="30"/>
       <c r="B51" s="4" t="s">
         <v>176</v>
       </c>
@@ -4856,13 +5014,13 @@
       <c r="A52" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="33" t="s">
-        <v>176</v>
-      </c>
-      <c r="C52" s="20" t="s">
+      <c r="B52" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="C52" s="27" t="s">
         <v>269</v>
       </c>
-      <c r="D52" s="20" t="s">
+      <c r="D52" s="27" t="s">
         <v>268</v>
       </c>
     </row>
@@ -4870,57 +5028,57 @@
       <c r="A53" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="27"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B54" s="33"/>
-      <c r="C54" s="20"/>
-      <c r="D54" s="20"/>
+      <c r="B54" s="31"/>
+      <c r="C54" s="27"/>
+      <c r="D54" s="27"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="B55" s="33"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
+      <c r="B55" s="31"/>
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B56" s="33"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="20"/>
+      <c r="B56" s="31"/>
+      <c r="C56" s="27"/>
+      <c r="D56" s="27"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B57" s="33"/>
-      <c r="C57" s="20"/>
-      <c r="D57" s="20"/>
+      <c r="B57" s="31"/>
+      <c r="C57" s="27"/>
+      <c r="D57" s="27"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B58" s="33"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="20"/>
+      <c r="B58" s="31"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="27"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="B59" s="33"/>
-      <c r="C59" s="20"/>
-      <c r="D59" s="20"/>
+      <c r="B59" s="31"/>
+      <c r="C59" s="27"/>
+      <c r="D59" s="27"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
@@ -4929,10 +5087,10 @@
       <c r="B60" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C60" s="20" t="s">
+      <c r="C60" s="27" t="s">
         <v>271</v>
       </c>
-      <c r="D60" s="20" t="s">
+      <c r="D60" s="27" t="s">
         <v>272</v>
       </c>
     </row>
@@ -4943,8 +5101,8 @@
       <c r="B61" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C61" s="20"/>
-      <c r="D61" s="20"/>
+      <c r="C61" s="27"/>
+      <c r="D61" s="27"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
@@ -4953,8 +5111,8 @@
       <c r="B62" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C62" s="20"/>
-      <c r="D62" s="20"/>
+      <c r="C62" s="27"/>
+      <c r="D62" s="27"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
@@ -4963,8 +5121,8 @@
       <c r="B63" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C63" s="20"/>
-      <c r="D63" s="20"/>
+      <c r="C63" s="27"/>
+      <c r="D63" s="27"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
@@ -4973,8 +5131,8 @@
       <c r="B64" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C64" s="20"/>
-      <c r="D64" s="20"/>
+      <c r="C64" s="27"/>
+      <c r="D64" s="27"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
@@ -4983,8 +5141,8 @@
       <c r="B65" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C65" s="20"/>
-      <c r="D65" s="20"/>
+      <c r="C65" s="27"/>
+      <c r="D65" s="27"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
@@ -4993,8 +5151,8 @@
       <c r="B66" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C66" s="20"/>
-      <c r="D66" s="20"/>
+      <c r="C66" s="27"/>
+      <c r="D66" s="27"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
@@ -5003,8 +5161,8 @@
       <c r="B67" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C67" s="20"/>
-      <c r="D67" s="20"/>
+      <c r="C67" s="27"/>
+      <c r="D67" s="27"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
@@ -5013,8 +5171,8 @@
       <c r="B68" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C68" s="20"/>
-      <c r="D68" s="20"/>
+      <c r="C68" s="27"/>
+      <c r="D68" s="27"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
@@ -5023,8 +5181,8 @@
       <c r="B69" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C69" s="20"/>
-      <c r="D69" s="20"/>
+      <c r="C69" s="27"/>
+      <c r="D69" s="27"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
@@ -5033,8 +5191,8 @@
       <c r="B70" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C70" s="20"/>
-      <c r="D70" s="20"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="27"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
@@ -5043,8 +5201,8 @@
       <c r="B71" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C71" s="20"/>
-      <c r="D71" s="20"/>
+      <c r="C71" s="27"/>
+      <c r="D71" s="27"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
@@ -5053,8 +5211,8 @@
       <c r="B72" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C72" s="20"/>
-      <c r="D72" s="20"/>
+      <c r="C72" s="27"/>
+      <c r="D72" s="27"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
@@ -5063,8 +5221,8 @@
       <c r="B73" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C73" s="20"/>
-      <c r="D73" s="20"/>
+      <c r="C73" s="27"/>
+      <c r="D73" s="27"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
@@ -5073,8 +5231,8 @@
       <c r="B74" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C74" s="20"/>
-      <c r="D74" s="20"/>
+      <c r="C74" s="27"/>
+      <c r="D74" s="27"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
@@ -5083,8 +5241,8 @@
       <c r="B75" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C75" s="20"/>
-      <c r="D75" s="20"/>
+      <c r="C75" s="27"/>
+      <c r="D75" s="27"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
@@ -5093,8 +5251,8 @@
       <c r="B76" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C76" s="20"/>
-      <c r="D76" s="20"/>
+      <c r="C76" s="27"/>
+      <c r="D76" s="27"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
@@ -5103,8 +5261,8 @@
       <c r="B77" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C77" s="20"/>
-      <c r="D77" s="20"/>
+      <c r="C77" s="27"/>
+      <c r="D77" s="27"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
@@ -5113,8 +5271,8 @@
       <c r="B78" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
+      <c r="C78" s="27"/>
+      <c r="D78" s="27"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
@@ -5123,8 +5281,8 @@
       <c r="B79" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C79" s="20"/>
-      <c r="D79" s="20"/>
+      <c r="C79" s="27"/>
+      <c r="D79" s="27"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
@@ -5133,8 +5291,8 @@
       <c r="B80" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C80" s="20"/>
-      <c r="D80" s="20"/>
+      <c r="C80" s="27"/>
+      <c r="D80" s="27"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
@@ -5143,8 +5301,8 @@
       <c r="B81" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C81" s="20"/>
-      <c r="D81" s="20"/>
+      <c r="C81" s="27"/>
+      <c r="D81" s="27"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
@@ -5153,8 +5311,8 @@
       <c r="B82" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C82" s="20"/>
-      <c r="D82" s="20"/>
+      <c r="C82" s="27"/>
+      <c r="D82" s="27"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
@@ -5163,8 +5321,8 @@
       <c r="B83" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C83" s="20"/>
-      <c r="D83" s="20"/>
+      <c r="C83" s="27"/>
+      <c r="D83" s="27"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
@@ -5173,8 +5331,8 @@
       <c r="B84" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C84" s="20"/>
-      <c r="D84" s="20"/>
+      <c r="C84" s="27"/>
+      <c r="D84" s="27"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
@@ -5183,8 +5341,8 @@
       <c r="B85" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C85" s="20"/>
-      <c r="D85" s="20"/>
+      <c r="C85" s="27"/>
+      <c r="D85" s="27"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
@@ -5193,8 +5351,8 @@
       <c r="B86" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C86" s="20"/>
-      <c r="D86" s="20"/>
+      <c r="C86" s="27"/>
+      <c r="D86" s="27"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
@@ -5203,8 +5361,8 @@
       <c r="B87" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C87" s="20"/>
-      <c r="D87" s="20"/>
+      <c r="C87" s="27"/>
+      <c r="D87" s="27"/>
     </row>
     <row r="88" spans="1:4" ht="120" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
@@ -5249,7 +5407,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A91" s="27" t="s">
+      <c r="A91" s="34" t="s">
         <v>283</v>
       </c>
       <c r="B91" s="4" t="s">
@@ -5263,7 +5421,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A92" s="27"/>
+      <c r="A92" s="34"/>
       <c r="B92" s="4" t="s">
         <v>176</v>
       </c>
@@ -5293,10 +5451,10 @@
         <v>68</v>
       </c>
       <c r="B94" s="4"/>
-      <c r="C94" s="20" t="s">
+      <c r="C94" s="27" t="s">
         <v>308</v>
       </c>
-      <c r="D94" s="20" t="s">
+      <c r="D94" s="27" t="s">
         <v>309</v>
       </c>
     </row>
@@ -5305,88 +5463,88 @@
         <v>69</v>
       </c>
       <c r="B95" s="4"/>
-      <c r="C95" s="20"/>
-      <c r="D95" s="20"/>
+      <c r="C95" s="27"/>
+      <c r="D95" s="27"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B96" s="4"/>
-      <c r="C96" s="20"/>
-      <c r="D96" s="20"/>
+      <c r="C96" s="27"/>
+      <c r="D96" s="27"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B97" s="4"/>
-      <c r="C97" s="20"/>
-      <c r="D97" s="20"/>
+      <c r="C97" s="27"/>
+      <c r="D97" s="27"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B98" s="4"/>
-      <c r="C98" s="20"/>
-      <c r="D98" s="20"/>
+      <c r="C98" s="27"/>
+      <c r="D98" s="27"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B99" s="4"/>
-      <c r="C99" s="20"/>
-      <c r="D99" s="20"/>
+      <c r="C99" s="27"/>
+      <c r="D99" s="27"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B100" s="4"/>
-      <c r="C100" s="20"/>
-      <c r="D100" s="20"/>
+      <c r="C100" s="27"/>
+      <c r="D100" s="27"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B101" s="4"/>
-      <c r="C101" s="20"/>
-      <c r="D101" s="20"/>
+      <c r="C101" s="27"/>
+      <c r="D101" s="27"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B102" s="4"/>
-      <c r="C102" s="20"/>
-      <c r="D102" s="20"/>
+      <c r="C102" s="27"/>
+      <c r="D102" s="27"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>77</v>
       </c>
       <c r="B103" s="4"/>
-      <c r="C103" s="20"/>
-      <c r="D103" s="20"/>
+      <c r="C103" s="27"/>
+      <c r="D103" s="27"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B104" s="4"/>
-      <c r="C104" s="20"/>
-      <c r="D104" s="20"/>
+      <c r="C104" s="27"/>
+      <c r="D104" s="27"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B105" s="4"/>
-      <c r="C105" s="20"/>
-      <c r="D105" s="20"/>
+      <c r="C105" s="27"/>
+      <c r="D105" s="27"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="15" t="s">
@@ -5395,10 +5553,10 @@
       <c r="B106" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C106" s="20" t="s">
+      <c r="C106" s="27" t="s">
         <v>310</v>
       </c>
-      <c r="D106" s="20" t="s">
+      <c r="D106" s="27" t="s">
         <v>311</v>
       </c>
     </row>
@@ -5409,8 +5567,8 @@
       <c r="B107" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C107" s="20"/>
-      <c r="D107" s="20"/>
+      <c r="C107" s="27"/>
+      <c r="D107" s="27"/>
     </row>
     <row r="108" spans="1:4" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="15" t="s">
@@ -5419,8 +5577,8 @@
       <c r="B108" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="C108" s="20"/>
-      <c r="D108" s="20"/>
+      <c r="C108" s="27"/>
+      <c r="D108" s="27"/>
     </row>
     <row r="109" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
@@ -5464,19 +5622,79 @@
         <v>331</v>
       </c>
     </row>
+    <row r="112" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C112" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="D112" s="8" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A113" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C113" s="27" t="s">
+        <v>383</v>
+      </c>
+      <c r="D113" s="27" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A114" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C114" s="27"/>
+      <c r="D114" s="27"/>
+    </row>
+    <row r="115" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C115" s="27" t="s">
+        <v>386</v>
+      </c>
+      <c r="D115" s="27" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A116" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C116" s="27"/>
+      <c r="D116" s="27"/>
+    </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="B52:B59"/>
-    <mergeCell ref="C52:C59"/>
-    <mergeCell ref="D52:D59"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="D13:D15"/>
+  <mergeCells count="32">
+    <mergeCell ref="C113:C114"/>
+    <mergeCell ref="D113:D114"/>
+    <mergeCell ref="C115:C116"/>
+    <mergeCell ref="D115:D116"/>
+    <mergeCell ref="C94:C105"/>
+    <mergeCell ref="D94:D105"/>
+    <mergeCell ref="C106:C108"/>
+    <mergeCell ref="D106:D108"/>
+    <mergeCell ref="A91:A92"/>
     <mergeCell ref="C60:C87"/>
     <mergeCell ref="D60:D87"/>
     <mergeCell ref="D18:D19"/>
@@ -5489,11 +5707,17 @@
     <mergeCell ref="D25:D27"/>
     <mergeCell ref="A20:A24"/>
     <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C94:C105"/>
-    <mergeCell ref="D94:D105"/>
-    <mergeCell ref="C106:C108"/>
-    <mergeCell ref="D106:D108"/>
-    <mergeCell ref="A91:A92"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B52:B59"/>
+    <mergeCell ref="C52:C59"/>
+    <mergeCell ref="D52:D59"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="D13:D15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5538,7 +5762,7 @@
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="34" t="s">
+      <c r="E3" s="35" t="s">
         <v>363</v>
       </c>
       <c r="F3" s="19" t="s">
@@ -5550,7 +5774,7 @@
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="34"/>
+      <c r="E4" s="35"/>
       <c r="F4" s="19" t="s">
         <v>350</v>
       </c>
@@ -5560,7 +5784,7 @@
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="35"/>
       <c r="F5" s="19" t="s">
         <v>351</v>
       </c>
@@ -5570,7 +5794,7 @@
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="34"/>
+      <c r="E6" s="35"/>
       <c r="F6" s="19" t="s">
         <v>352</v>
       </c>
@@ -5580,7 +5804,7 @@
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="34"/>
+      <c r="E7" s="35"/>
       <c r="F7" s="19" t="s">
         <v>353</v>
       </c>
@@ -5590,7 +5814,7 @@
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="34"/>
+      <c r="E8" s="35"/>
       <c r="F8" s="19" t="s">
         <v>355</v>
       </c>
@@ -5600,7 +5824,7 @@
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="34"/>
+      <c r="E9" s="35"/>
       <c r="F9" s="19" t="s">
         <v>354</v>
       </c>
@@ -5610,7 +5834,7 @@
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="34"/>
+      <c r="E10" s="35"/>
       <c r="F10" s="19" t="s">
         <v>356</v>
       </c>
@@ -5620,7 +5844,7 @@
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="36" t="s">
         <v>364</v>
       </c>
       <c r="F11" s="19" t="s">
@@ -5632,7 +5856,7 @@
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="35"/>
+      <c r="E12" s="36"/>
       <c r="F12" s="19" t="s">
         <v>359</v>
       </c>
@@ -5642,7 +5866,7 @@
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="35"/>
+      <c r="E13" s="36"/>
       <c r="F13" s="19" t="s">
         <v>360</v>
       </c>
@@ -5652,7 +5876,7 @@
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="35"/>
+      <c r="E14" s="36"/>
       <c r="F14" s="19" t="s">
         <v>358</v>
       </c>
@@ -5662,7 +5886,7 @@
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="35"/>
+      <c r="E15" s="36"/>
       <c r="F15" s="19" t="s">
         <v>361</v>
       </c>
@@ -5672,7 +5896,7 @@
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="35"/>
+      <c r="E16" s="36"/>
       <c r="F16" s="19" t="s">
         <v>362</v>
       </c>

</xml_diff>